<commit_message>
Reschedule Monday and Friday lessons for grades 7 and 10
</commit_message>
<xml_diff>
--- a/Расписание уроков .xlsx
+++ b/Расписание уроков .xlsx
@@ -1445,13 +1445,13 @@
         <v>27</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="O3" s="8" t="s">
         <v>29</v>
       </c>
       <c r="P3" s="9" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="Q3" s="10">
         <v>1.0</v>
@@ -1555,13 +1555,13 @@
         <v>39</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="O5" s="15" t="s">
         <v>47</v>
       </c>
       <c r="P5" s="9" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="Q5" s="19">
         <v>3.0</v>
@@ -1608,7 +1608,7 @@
         <v>40</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="O6" s="15" t="s">
         <v>30</v>
@@ -1667,7 +1667,7 @@
         <v>41</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>47</v>
+        <v>121</v>
       </c>
       <c r="Q7" s="24">
         <v>5.0</v>
@@ -1734,9 +1734,7 @@
       <c r="M9" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="N9" s="15" t="s">
-        <v>63</v>
-      </c>
+      <c r="N9" s="15"/>
       <c r="O9" s="15" t="s">
         <v>40</v>
       </c>
@@ -2937,7 +2935,7 @@
         <v>120</v>
       </c>
       <c r="P35" s="8" t="s">
-        <v>121</v>
+        <v>47</v>
       </c>
       <c r="Q35" s="10">
         <v>1.0</v>
@@ -2988,7 +2986,7 @@
         <v>124</v>
       </c>
       <c r="N36" s="15" t="s">
-        <v>125</v>
+        <v>47</v>
       </c>
       <c r="O36" s="53" t="s">
         <v>26</v>
@@ -3187,7 +3185,9 @@
       <c r="M40" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="N40" s="30"/>
+      <c r="N40" s="30" t="s">
+        <v>63</v>
+      </c>
       <c r="O40" s="53" t="s">
         <v>40</v>
       </c>

</xml_diff>

<commit_message>
Move grade 8 informatics to Friday without teacher gaps
</commit_message>
<xml_diff>
--- a/Расписание уроков .xlsx
+++ b/Расписание уроков .xlsx
@@ -1447,8 +1447,10 @@
       <c r="N3" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="O3" s="8" t="s">
-        <v>29</v>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Русс.язык</t>
+        </is>
       </c>
       <c r="P3" s="9" t="s">
         <v>48</v>
@@ -1557,8 +1559,10 @@
       <c r="N5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="O5" s="15" t="s">
-        <v>47</v>
+      <c r="O5" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">История </t>
+        </is>
       </c>
       <c r="P5" s="9" t="s">
         <v>30</v>
@@ -1735,8 +1739,10 @@
         <v>65</v>
       </c>
       <c r="N9" s="15"/>
-      <c r="O9" s="15" t="s">
-        <v>40</v>
+      <c r="O9" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Литература </t>
+        </is>
       </c>
       <c r="P9" s="36"/>
       <c r="Q9" s="37">
@@ -2988,8 +2994,10 @@
       <c r="N36" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="O36" s="53" t="s">
-        <v>26</v>
+      <c r="O36" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">География </t>
+        </is>
       </c>
       <c r="P36" s="15" t="s">
         <v>41</v>
@@ -3041,8 +3049,10 @@
       <c r="N37" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="O37" s="53" t="s">
-        <v>30</v>
+      <c r="O37" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Информатика</t>
+        </is>
       </c>
       <c r="P37" s="15" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
Set grade 10 Friday first lesson to literature without teacher gaps
</commit_message>
<xml_diff>
--- a/Расписание уроков .xlsx
+++ b/Расписание уроков .xlsx
@@ -2940,8 +2940,10 @@
       <c r="O35" s="53" t="s">
         <v>120</v>
       </c>
-      <c r="P35" s="8" t="s">
-        <v>47</v>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Литература </t>
+        </is>
       </c>
       <c r="Q35" s="10">
         <v>1.0</v>
@@ -2996,11 +2998,13 @@
       </c>
       <c r="O36" s="53" t="inlineStr">
         <is>
-          <t xml:space="preserve">География </t>
+          <t xml:space="preserve">Геометрия </t>
         </is>
       </c>
-      <c r="P36" s="15" t="s">
-        <v>41</v>
+      <c r="P36" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Русс.язык</t>
+        </is>
       </c>
       <c r="Q36" s="17">
         <v>2.0</v>
@@ -3043,8 +3047,10 @@
       <c r="L37" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="M37" s="56" t="s">
-        <v>128</v>
+      <c r="M37" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Русс.яз </t>
+        </is>
       </c>
       <c r="N37" s="15" t="s">
         <v>41</v>
@@ -3107,8 +3113,10 @@
       <c r="O38" s="53" t="s">
         <v>130</v>
       </c>
-      <c r="P38" s="15" t="s">
-        <v>26</v>
+      <c r="P38" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Информатика</t>
+        </is>
       </c>
       <c r="Q38" s="22">
         <v>4.0</v>
@@ -3157,11 +3165,15 @@
       <c r="N39" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="O39" s="53" t="s">
-        <v>48</v>
-      </c>
-      <c r="P39" s="15" t="s">
-        <v>30</v>
+      <c r="O39" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">География </t>
+        </is>
+      </c>
+      <c r="P39" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Алгебра </t>
+        </is>
       </c>
       <c r="Q39" s="24">
         <v>5.0</v>
@@ -3192,8 +3204,10 @@
       <c r="L40" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="M40" s="56" t="s">
-        <v>46</v>
+      <c r="M40" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ОФП/ИЗО/Труд</t>
+        </is>
       </c>
       <c r="N40" s="30" t="s">
         <v>63</v>

</xml_diff>